<commit_message>
docs(order-management): lock 24.7 scope — GET payments only, write side covered by 24.8, both open questions resolved
</commit_message>
<xml_diff>
--- a/order_management/24.7-manual-payment-methods/24.7 - Manual Payment Methods.xlsx
+++ b/order_management/24.7-manual-payment-methods/24.7 - Manual Payment Methods.xlsx
@@ -24,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -43,8 +43,12 @@
       <color rgb="000563C1"/>
       <u val="single"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -81,8 +85,13 @@
         <fgColor rgb="001F4E78"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1F4E78"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -104,11 +113,25 @@
         <color rgb="00BFBFBF"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFBFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFBFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFBFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFBFBFBF"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -147,6 +170,15 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -563,7 +595,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>5 requirement(s) to implement here (filter Build Focus = 'Implement here'). 0 covered elsewhere, 0 out of scope.</t>
+          <t>Scope locked 2026-07-03 (Step-1 gate complete). 2 to implement here, 3 covered elsewhere (by 24.8), 0 out of scope. Release model: ship-together, builds after 24.8.</t>
         </is>
       </c>
     </row>
@@ -573,8 +605,10 @@
           <t>To implement here</t>
         </is>
       </c>
-      <c r="B5" s="3" t="n">
-        <v>5</v>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
     </row>
     <row r="6" ht="80" customHeight="1">
@@ -585,13 +619,21 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Story 24.7 asks Admin to treat Bank Wire, ACH, PayPal and Check as manual payment methods and to manually mark such payments Paid or Unpaid from the admin panel, with status changes logged and enforced server-side. Re-verification against code confirms the building blocks but not the feature: the manual-method taxonomy is the CartPaymentMethod enum (credit_card, bank_wire_ach, check, paypal) and it IS actually written — cart-payment-plan.service.upsertPlan persists entries.method — but only on the cart's payment plan, which the schema marks "display only — no charging," and the Order model has NO payment_method column (verified: grep returns nothing; checkout.service never copies a method onto the order). Order.status (OrderStatus enum) is writable (order.update precedent in ppl-order) and the AdminAuditService with entity_type=order is fully built and already used in checkout, so a net-new admin endpoint that sets status and logs it is Deliverable. The two partial pieces are: (a) no order-level field classifies an order as manual vs Stripe (derivable from cart-&gt;plan-&gt;entries.method for product orders only; subscription/ppl_addon orders have no cart and are Stripe-only), and (d) the method-eligibility gate depends on that classification. OrderStatus also has no native Paid/Unpaid values, so they must be mapped or added. Overall feasible as a net-new Order Management endpoint.</t>
+          <t>Story converged to least-work shape: ONE read route (GET :id/payments via 24.8's mapper, incl. per-installment payment_memo + derived Paid/Unpaid label); write side (mark Paid/Unpaid + logging + enforcement) delivered by 24.8's installment PATCH; planned PATCH :id/payment-status DROPPED (D3); classification = 24.8's payment_type; both open questions resolved (derive-not-store; restrict-to-manual per-installment).</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="inlineStr"/>
-      <c r="B7" s="2" t="inlineStr"/>
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>Covered Elsewhere</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>3 (24.7-b/c/d -&gt; 24.8)</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
@@ -610,7 +652,7 @@
         </is>
       </c>
       <c r="B9" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10">
@@ -620,7 +662,7 @@
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -661,7 +703,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Not started — analysis only</t>
+          <t>Not started — scope locked 2026-07-03 (gate complete)</t>
         </is>
       </c>
     </row>
@@ -787,7 +829,7 @@
       </c>
       <c r="L1" s="9" t="inlineStr">
         <is>
-          <t>Impl Status (2026-07-01)</t>
+          <t>Impl Status (2026-07-03)</t>
         </is>
       </c>
     </row>
@@ -804,7 +846,7 @@
       </c>
       <c r="C2" s="10" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Deliverable</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
@@ -812,22 +854,22 @@
           <t>Implement here</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>The manual-method taxonomy is modeled AND written: CartPaymentMethod enum (credit_card, bank_wire_ach, check, paypal) and cart-payment-plan.service.upsertPlan actually persists entries.method, so this is a real written producer, not a dead column. BUT it lives only on CartPaymentScheduleEntry as part of the cart's payment plan, which the schema explicitly marks 'Persisted for validation/display only — no charging happens here.' The Order model has NO payment_method column (verified by grep) and checkout.service never copies a method onto the order. For product orders the manual method is derivable today via cart_id-&gt;CartPaymentPlan-&gt;entries.method; subscription/ppl_addon orders have no cart and are always Stripe. So building requires adding an order-level method field or a documented derivation; the data primitive exists and is populated for product orders, hence Partial not Blocked.</t>
+          <t>CONFIRMED 2026-07-03 — upgraded Partial -&gt; Deliverable (sequenced on 24.8's migration). Classification source of record = payment_type on payment_transactions (24.8 D2: CartPaymentMethod reuse — exactly this taxonomy, bank_wire_ach = Bank Wire + ACH; doc-comment: credit_card = Stripe card charge, sole non-manual). 'Treated as manual' = locked behaviors elsewhere: excluded from charge cron (24.8 D3 guard), hand-markable (24.8-c gate), Manual-refund-only without charge id (24.9-f), classified via the mapper. Historic rows credit_card via backfill (all 5 creation sites verified card flows); subscription/ppl_addon always-Stripe; no cart-plan fallback needed.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>admin-backend-api/prisma/schema.prisma:2753 (CartPaymentMethod enum); schema.prisma:2837-2868 (CartPaymentScheduleEntry.method, 'display only'); admin-backend-api/src/admin/cart/services/cart-payment-plan.service.ts:85-96 (upsert writes entries.method); schema.prisma:1540-1604 (Order model — no payment_method field, confirmed)</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr"/>
+          <t>24.8 doc D2/D3 locked 2026-07-03; admin schema CartPaymentMethod :2801-2808; cart-payment-plan.service.ts:95 (intent writer, display-only :2909-2910); Order has no payment_method :1541-1609 (correct — per-installment)</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>24.8 (SBE-1132) payment_type migration — same release, builds first</t>
+        </is>
+      </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
           <t>[C13 cross-reference] Mostly delivered by building 24.8 (A single PaymentTransaction -&gt; installment-row mapper (Invo…). Residual: the Payments screen reuses the installment row projection but focuses on status/method; catalog deliberately keeps GET .../payments a DISTINCT endpoint from GET .../payment-plan. No endpoint merge — only the row mapper is shared.</t>
@@ -845,7 +887,7 @@
       </c>
       <c r="L2" s="12" t="inlineStr">
         <is>
-          <t>◻ Not started</t>
+          <t>Gate 2026-07-03: upgraded Partial -&gt; Deliverable (sequenced on 24.8).</t>
         </is>
       </c>
     </row>
@@ -862,30 +904,34 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Deliverable</t>
+          <t>Covered elsewhere</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Implement here</t>
+          <t>Covered elsewhere</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>24.8 (SBE-1132) — installment PATCH</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Buildable as a net-new admin endpoint on built primitives: the Order model and OrderStatus enum (pending/partially_paid/completed/failed/refunded/canceled) exist, and prisma order.update is already used in admin (ppl-order billing update at :175). 'Paid'/'Unpaid' must be mapped onto existing OrderStatus values (e.g. completed/pending) or a new value/flag added, since OrderStatus has no native Paid/Unpaid. No Order Management module/controller exists yet, so the endpoint is net-new. Today Order.status transitions are owned exclusively by the Stripe webhook handler (computeNewOrderStatus / syncOrderOnInvoicePaid), so this introduces an admin-owned write-path that must coexist with webhook ownership for non-manual orders.</t>
+          <t>CONFIRMED 2026-07-03. Delivered entirely by 24.8's PATCH :id/payment-plan/installments/:installmentId, locked with exactly this row's semantics: manual-method-only eligibility, Paid =&gt; succeeded + paid_at + webhook-mirroring money writes, Unpaid =&gt; scheduled + bookkeeping reversal, label derived. OLD OQ-1 RESOLVED derive-not-store (neither OrderStatus overload nor new field). 24.7 builds no write path (D3: planned order-level PATCH dropped).</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>admin-backend-api/prisma/schema.prisma:421-430 (OrderStatus enum); admin-backend-api/src/admin/ppl-order/ppl-order.service.ts:175 (order.update precedent, billing only); external-api-service/src/modules/webhook/services/webhook.service.ts:677,2245-2253 (webhook owns paid/completed transitions)</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr"/>
+          <t>24.8 doc 24.8-c locked; ext webhook.service.ts:2114-2125/:2281-2287 (mirrored writes); exh orders.helpers.ts:53</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>— delivered by 24.8, same release</t>
+        </is>
+      </c>
       <c r="I3" s="2" t="inlineStr"/>
       <c r="J3" s="2" t="inlineStr">
         <is>
@@ -899,7 +945,7 @@
       </c>
       <c r="L3" s="12" t="inlineStr">
         <is>
-          <t>◻ Not started</t>
+          <t>Gate 2026-07-03: reclassified Deliverable -&gt; Covered elsewhere (24.8).</t>
         </is>
       </c>
     </row>
@@ -916,30 +962,34 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Deliverable</t>
+          <t>Covered elsewhere</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Implement here</t>
+          <t>Covered elsewhere</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>24.8 (SBE-1132) — PATCH audit leg</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Fully supported by built primitives. AdminAuditService.record/recordMany write append-only audit rows, AdminAuditEntityType already includes 'order', and that entity type is already used in the checkout flow. The new status-update service call wraps a record() in the same transaction (previous_value=old status, new_value=new status, performedBy=admin id).</t>
+          <t>CONFIRMED 2026-07-03. Logging = AdminAuditService.record() inside 24.8's PATCH tx (old-&gt;new status, admin id, non-blank note); shipped in-module precedent from 24.14 (order-notes.service.ts:94). 'Refer 24.14' pointer satisfied by the shipped audit-log read endpoint. 24.7's own route is a read — logs nothing.</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>admin-backend-api/src/admin/common/audit/admin-audit.service.ts:30-49; schema.prisma:2193 (AdminAuditEntityType.order); admin-backend-api/src/admin/cart/services/checkout.service.ts:329 (AdminAuditEntityType.order already in use)</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="inlineStr"/>
+          <t>admin admin-audit.service.ts:30/:50; order-notes.service.ts:94; schema :2210</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>— delivered by 24.8, same release</t>
+        </is>
+      </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
           <t>[C9 build-once-reuse] Mostly delivered by building 24.14 (AdminAuditService.record()/recordMany() with entity_type='o…). Residual: one record() call inside the payment-status transaction.</t>
@@ -957,7 +1007,7 @@
       </c>
       <c r="L4" s="12" t="inlineStr">
         <is>
-          <t>◻ Not started</t>
+          <t>Gate 2026-07-03: reclassified -&gt; Covered elsewhere (24.8).</t>
         </is>
       </c>
     </row>
@@ -974,30 +1024,34 @@
       </c>
       <c r="C5" s="10" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Covered elsewhere</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Implement here</t>
+          <t>Covered elsewhere</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>24.8 (SBE-1132) — gate + route enforcement</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Server-side enforcement scaffolding is built: the @Permissions guard + DTO validation pattern is used across admin controllers (e.g. ppl-order.controller @Permissions('ppl-order.update') on a @Patch(':id')), so requiring a permission and validating the payload is Deliverable. The missing piece is the method-specific gate — 'only manual-method (Bank Wire/ACH/PayPal/Check) orders may be marked Paid/Unpaid, credit-card orders stay webhook-driven' — which cannot be enforced because no order-level field identifies an order as manual (see 24.7-a). Without that classification the backend cannot reliably distinguish eligible orders for non-cart orders.</t>
+          <t>CONFIRMED 2026-07-03 — upgraded Partial -&gt; Covered elsewhere. Both halves locked into 24.8: method-eligibility gate (manual-only, per-installment via payment_type — handles mixed plans; OLD OQ-2 RESOLVED restrict-to-manual, no admin override on card rows) and permission/DTO enforcement on the PATCH (orders.payment-plan.* key). 24.7's residual = its read route's permission (rides 24.7-e).</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>admin-backend-api/src/admin/ppl-order/ppl-order.controller.ts:129-130 (@Permissions guard + @Patch(':id') pattern); schema.prisma:1540-1604 (Order lacks payment_method to gate on); external-api-service/src/modules/webhook/services/webhook.service.ts:2245-2253 (status transitions today owned by webhook)</t>
-        </is>
-      </c>
-      <c r="H5" s="2" t="inlineStr"/>
+          <t>24.8 doc 24.8-c/D3 locked; orders.controller.ts:51/:95/:132 (@Permissions in-module precedent)</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>— delivered by 24.8, same release</t>
+        </is>
+      </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
           <t>[C8 build-once-reuse] Mostly delivered by building 24.1 (The existing JWT + roles guard + @Permissions(...) decorato…). Residual: the method-eligibility gate (manual-method-only) is extra DOMAIN logic on top of the shared guard (24.7-d is Partial for that reason).</t>
@@ -1015,7 +1069,7 @@
       </c>
       <c r="L5" s="12" t="inlineStr">
         <is>
-          <t>◻ Not started</t>
+          <t>Gate 2026-07-03: upgraded Partial -&gt; Covered elsewhere (24.8).</t>
         </is>
       </c>
     </row>
@@ -1040,22 +1094,22 @@
           <t>Implement here</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>A read endpoint returning order payment status is buildable on existing populated data: Order.status, paid_amount, paid_in_full_at and payment_transactions are all populated, and an existing precedent derives a human payment_status_label from Order.status (ppl-order). Net-new since no Order Management controller exists. The displayed 'payment method' value depends on the same missing order-level method field as 24.7-a — confirmed by the existing ppl-order detail view which HARDCODES payment.payment_type = 'Credit Card' because no per-order method exists — but the status/amounts read view itself is fully deliverable.</t>
+          <t>CONFIRMED 2026-07-03 — THE WHOLE OF 24.7'S BUILD. GET /api/v1/orders/:id/payments: additive route on the shipped module (no payments route anywhere in admin src); installment rows via 24.8's C13 mapper (status, amounts, dates, Invoice #, payment_type, per-installment payment_memo per D3 rider) + order money summary (paid_amount, paid_in_full_at, derived Paid/Unpaid label — deriveOrderPaymentStatus port). DISTINCT from GET :id/payment-plan (same mapper, different lens). Residuals: orders.payments.read seed + Swagger. The old ppl-order hardcoded payment_type 'Credit Card' (:378) is exactly what payment_type retires.</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>admin-backend-api/src/admin/ppl-order/ppl-order.service.ts:345,359 (payment_status_label derivation); ppl-order.service.ts (payment.payment_type hardcoded 'Credit Card'); schema.prisma:1573-1574 (paid_amount, paid_in_full_at); schema.prisma:2056-2091 (PaymentTransaction)</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="inlineStr"/>
+          <t>orders.controller.ts routes :50/:94/:131 only; schema paid_amount :1578, paid_in_full_at :1579, PT :2073-2108; exh orders.helpers.ts:53/:74; ppl-order.service.ts:345/:359/:378</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>24.8 (SBE-1132) C13 mapper — same release, builds first</t>
+        </is>
+      </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
           <t>[C13 cross-reference] Mostly delivered by building 24.8 (A single PaymentTransaction -&gt; installment-row mapper (Invo…). Residual: the Payments screen reuses the installment row projection but focuses on status/method; catalog deliberately keeps GET .../payments a DISTINCT endpoint from GET .../payment-plan. No endpoint merge — only the row mapper is shared.</t>
@@ -1073,7 +1127,7 @@
       </c>
       <c r="L6" s="12" t="inlineStr">
         <is>
-          <t>◻ Not started</t>
+          <t>Gate 2026-07-03: Deliverable (sequenced on 24.8 mapper).</t>
         </is>
       </c>
     </row>
@@ -1136,48 +1190,56 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>PATCH</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>/api/v1/orders/:id/payment-status</t>
+          <t>/api/v1/orders/:id/payments</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Admin manually sets a manual-method order's payment status to Paid or Unpaid; server-side validation, @Permissions check, method-eligibility gate, AdminAuditLog write in one transaction.</t>
+          <t>The Payments view: installment rows via 24.8's C13 mapper (incl. payment_type + per-installment payment_memo) + order money summary + derived Paid/Unpaid label. 24.7's ONLY route.</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>24.7-b, 24.7-c, 24.7-d</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr"/>
+          <t>24.7-a, 24.7-e</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Mapper owned by 24.8; distinct from GET :id/payment-plan by design</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>(dropped)</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>/api/v1/orders/:id/payments</t>
+          <t>PATCH /api/v1/orders/:id/payment-status — DROPPED 2026-07-03 (D3)</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>The order's Payments view (current paid/unpaid status, payment method, amounts, installment/transaction rows) backing the admin Payments screen.</t>
+          <t>Mark-as-Paid/Unpaid lives solely in 24.8's PATCH :id/payment-plan/installments/:installmentId — one writer, one audit trail, one permission surface.</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>24.7-a, 24.7-e</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr"/>
+          <t>24.7-b/c/d (delivered there)</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>24.8 owns</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1190,74 +1252,84 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="120" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
-    <col width="120" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="9" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B1" s="9" t="inlineStr">
-        <is>
-          <t>Open Question</t>
-        </is>
-      </c>
-      <c r="C1" s="9" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="D1" s="9" t="inlineStr">
-        <is>
-          <t>Resolution / Decision</t>
+      <c r="A1" s="14" t="inlineStr">
+        <is>
+          <t>Req</t>
+        </is>
+      </c>
+      <c r="B1" s="14" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="C1" s="14" t="inlineStr">
+        <is>
+          <t>Verdict</t>
+        </is>
+      </c>
+      <c r="D1" s="14" t="inlineStr">
+        <is>
+          <t>Open Question / What is needed</t>
+        </is>
+      </c>
+      <c r="E1" s="14" t="inlineStr">
+        <is>
+          <t>Dependency (blocking story + Jira)</t>
+        </is>
+      </c>
+      <c r="F1" s="14" t="inlineStr">
+        <is>
+          <t>Assignee</t>
+        </is>
+      </c>
+      <c r="G1" s="14" t="inlineStr">
+        <is>
+          <t>Sprint / Jira status</t>
+        </is>
+      </c>
+      <c r="H1" s="14" t="inlineStr">
+        <is>
+          <t>Decision / Current direction</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Should Paid/Unpaid map onto existing OrderStatus values (e.g. completed/pending) or be a new dedicated payment-state field/enum? OrderStatus today is pending/partially_paid/completed/failed/refunded/canceled with no native Paid/Unpaid.</t>
-        </is>
-      </c>
-      <c r="C2" s="12" t="inlineStr">
-        <is>
-          <t>OPEN — for team discussion</t>
-        </is>
-      </c>
-      <c r="D2" s="12" t="inlineStr">
-        <is>
-          <t>Current direction (2026-07-01): lean toward mapping Paid/Unpaid onto existing OrderStatus (completed = Paid; pending/partially_paid = Unpaid) to avoid a schema change; a dedicated payment-state field/enum remains under consideration. Pending team confirmation.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>For an order whose status is otherwise owned by the Stripe webhook (credit-card or split-installment orders), is manual marking strictly forbidden, or may an admin override? The cart payment plan supports per-entry methods, so mixed card+manual plans are representable and the coexistence rule with the webhook-owned status machine is unspecified.</t>
-        </is>
-      </c>
-      <c r="C3" s="12" t="inlineStr">
-        <is>
-          <t>OPEN — for team discussion</t>
-        </is>
-      </c>
-      <c r="D3" s="12" t="inlineStr">
-        <is>
-          <t>Current direction (2026-07-01): lean toward restricting manual marking to manual-method (Bank Wire/ACH/PayPal/Check) orders only, leaving credit-card/webhook-owned orders webhook-driven; mixed card+manual plan case unresolved. Pending team confirmation.</t>
+      <c r="A2" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B2" s="15" t="inlineStr">
+        <is>
+          <t>Register empty — gate locked 2026-07-03</t>
+        </is>
+      </c>
+      <c r="C2" s="15" t="inlineStr"/>
+      <c r="D2" s="15" t="inlineStr">
+        <is>
+          <t>OQ-1 (Paid/Unpaid representation) RESOLVED: derive-not-store — PT.status flip + webhook-mirroring money writes + derived label (24.8-c). OQ-2 (webhook coexistence) RESOLVED: restrict-to-manual per-installment via payment_type; card rows webhook-owned, no override; mixed plans handled per-installment.</t>
+        </is>
+      </c>
+      <c r="E2" s="15" t="inlineStr"/>
+      <c r="F2" s="15" t="inlineStr"/>
+      <c r="G2" s="15" t="inlineStr"/>
+      <c r="H2" s="15" t="inlineStr">
+        <is>
+          <t>2 Deliverable + 3 covered by 24.8; PATCH dropped (D3).</t>
         </is>
       </c>
     </row>
@@ -1272,7 +1344,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="55" customWidth="1" min="1" max="1"/>
@@ -1298,13 +1370,38 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr"/>
-      <c r="C2" s="2" t="inlineStr"/>
+      <c r="A2" s="15" t="inlineStr">
+        <is>
+          <t>payment_type/payment_memo columns, NOT-NULL relaxation, C13 mapper, installment PATCH (flip + audit + gate)</t>
+        </is>
+      </c>
+      <c r="B2" s="15" t="inlineStr">
+        <is>
+          <t>24.7-a, b, c, d, e</t>
+        </is>
+      </c>
+      <c r="C2" s="15" t="inlineStr">
+        <is>
+          <t>24.8 (SBE-1132) — same release, builds immediately before 24.7</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="15" t="inlineStr">
+        <is>
+          <t>Downstream readers (NOT dependencies): 24.15 stop-condition (PT.status at send time); 24.10-g (manual representation for cancel/refund marking)</t>
+        </is>
+      </c>
+      <c r="B3" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C3" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1317,7 +1414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1337,122 +1434,158 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="12" t="inlineStr">
+      <c r="A2" s="16" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="B2" s="12" t="inlineStr">
-        <is>
-          <t>Not started — analysis/feasibility stage only. No branch, no SBE ticket, no PR, no Swagger tag. All five in-scope requirements are ◻ Not started.</t>
+      <c r="B2" s="15" t="inlineStr">
+        <is>
+          <t>Not started — Step-1 gate complete 2026-07-03; scope locked (order-level PATCH dropped per D3; write side covered by 24.8; both old open questions resolved via 24.8-c). Release model: ship-together; builds after 24.8.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="12" t="inlineStr">
-        <is>
-          <t>Remaining — 24.7-a</t>
-        </is>
-      </c>
-      <c r="B3" s="12" t="inlineStr">
-        <is>
-          <t>Recognize/classify an order as manual vs Stripe; needs an order-level method field or a documented cart→plan→entries.method derivation (Partial per feasibility). ◻ Not started.</t>
+      <c r="A3" s="16" t="inlineStr">
+        <is>
+          <t>Branch</t>
+        </is>
+      </c>
+      <c r="B3" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="12" t="inlineStr">
-        <is>
-          <t>Remaining — 24.7-b</t>
-        </is>
-      </c>
-      <c r="B4" s="12" t="inlineStr">
-        <is>
-          <t>Net-new admin PATCH /orders/:id/payment-status setting Paid/Unpaid, coexisting with webhook-owned status. ◻ Not started.</t>
+      <c r="A4" s="16" t="inlineStr">
+        <is>
+          <t>SBE ticket</t>
+        </is>
+      </c>
+      <c r="B4" s="15" t="inlineStr">
+        <is>
+          <t>SBE-1131 (In Progress, Prantik Saha)</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="12" t="inlineStr">
-        <is>
-          <t>Remaining — 24.7-c</t>
-        </is>
-      </c>
-      <c r="B5" s="12" t="inlineStr">
-        <is>
-          <t>Log status changes via one AdminAuditService.record() inside the update transaction (entity_type=order). ◻ Not started.</t>
+      <c r="A5" s="16" t="inlineStr">
+        <is>
+          <t>Commits</t>
+        </is>
+      </c>
+      <c r="B5" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="12" t="inlineStr">
-        <is>
-          <t>Remaining — 24.7-d</t>
-        </is>
-      </c>
-      <c r="B6" s="12" t="inlineStr">
-        <is>
-          <t>Server-side enforcement: @Permissions guard + DTO validation + method-eligibility gate (depends on 24.7-a classification; Partial). ◻ Not started.</t>
+      <c r="A6" s="16" t="inlineStr">
+        <is>
+          <t>PR</t>
+        </is>
+      </c>
+      <c r="B6" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="12" t="inlineStr">
-        <is>
-          <t>Remaining — 24.7-e</t>
-        </is>
-      </c>
-      <c r="B7" s="12" t="inlineStr">
-        <is>
-          <t>GET /orders/:id/payments Payments read view (status/amounts/transactions); method value depends on the same missing order-level method field. ◻ Not started.</t>
+      <c r="A7" s="16" t="inlineStr">
+        <is>
+          <t>Swagger tag</t>
+        </is>
+      </c>
+      <c r="B7" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="12" t="inlineStr">
-        <is>
-          <t>Open decision — Paid/Unpaid representation</t>
-        </is>
-      </c>
-      <c r="B8" s="12" t="inlineStr">
-        <is>
-          <t>Map onto existing OrderStatus (completed/pending) or add a dedicated payment-state field/enum? Gates 24.7-b, 24.7-e. No code until answered.</t>
+      <c r="A8" s="16" t="inlineStr">
+        <is>
+          <t>Build gates</t>
+        </is>
+      </c>
+      <c r="B8" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="12" t="inlineStr">
-        <is>
-          <t>Open decision — webhook coexistence</t>
-        </is>
-      </c>
-      <c r="B9" s="12" t="inlineStr">
-        <is>
-          <t>For webhook-owned (credit-card/split-installment) orders, is manual marking forbidden or may an admin override? Gates 24.7-b, 24.7-d. No code until answered.</t>
+      <c r="A9" s="16" t="inlineStr">
+        <is>
+          <t>Live smoke</t>
+        </is>
+      </c>
+      <c r="B9" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="12" t="inlineStr">
-        <is>
-          <t>Dependencies</t>
-        </is>
-      </c>
-      <c r="B10" s="12" t="inlineStr">
-        <is>
-          <t>None — Cross-Epic Dependencies: None; no requirement delivered elsewhere (all Build Focus 'Implement here'). Build-once-reuse primitives (AdminAuditService, @Permissions guard, PaymentTransaction row mapper) are shared scaffolding, not blocking dependencies.</t>
+      <c r="A10" s="16" t="inlineStr">
+        <is>
+          <t>Confirmed build scope</t>
+        </is>
+      </c>
+      <c r="B10" s="15" t="inlineStr">
+        <is>
+          <t>GET /orders/:id/payments (C13 mapper reuse + per-installment payment_memo + derived Paid/Unpaid label) + orders.payments.read seed + Swagger registration</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="12" t="inlineStr">
+      <c r="A11" s="16" t="inlineStr">
+        <is>
+          <t>Remaining</t>
+        </is>
+      </c>
+      <c r="B11" s="15" t="inlineStr">
+        <is>
+          <t>The one route unbuilt</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="16" t="inlineStr">
+        <is>
+          <t>Not ready — see Open Questions</t>
+        </is>
+      </c>
+      <c r="B12" s="15" t="inlineStr">
+        <is>
+          <t>none — register empty</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="16" t="inlineStr">
+        <is>
+          <t>External dependencies — see Cross-Epic Dependencies</t>
+        </is>
+      </c>
+      <c r="B13" s="15" t="inlineStr">
+        <is>
+          <t>24.8 (mapper + payment_type + PATCH) — same release, builds first</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="16" t="inlineStr">
         <is>
           <t>Out of API scope</t>
         </is>
       </c>
-      <c r="B11" s="12" t="inlineStr">
-        <is>
-          <t>Front-end wiring (Payments screen, status-toggle UI).</t>
+      <c r="B14" s="15" t="inlineStr">
+        <is>
+          <t>Payments screen FE wiring, status-toggle UI</t>
         </is>
       </c>
     </row>

</xml_diff>